<commit_message>
forming and coding manual datasets
</commit_message>
<xml_diff>
--- a/data/manual_coding_dataset.xlsx
+++ b/data/manual_coding_dataset.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wikto\python_project\EU_leadership_docs\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81CA8428-BFDD-4612-B99E-4330AD099631}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8B9EFFF-A2FD-4D71-98EC-74B25806645D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="340" yWindow="340" windowWidth="13970" windowHeight="10450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DATA" sheetId="1" r:id="rId1"/>
@@ -1638,7 +1638,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="174" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>41740</v>
       </c>
@@ -1820,7 +1820,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="319" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" ht="333.5" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
         <v>41974</v>
       </c>
@@ -3039,7 +3039,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="60" spans="1:8" ht="145" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:8" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A60" s="1">
         <v>42620</v>
       </c>
@@ -4001,7 +4001,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="97" spans="1:8" ht="246.5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:8" ht="261" x14ac:dyDescent="0.35">
       <c r="A97" s="1">
         <v>43410</v>
       </c>
@@ -4131,7 +4131,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="102" spans="1:8" ht="261" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:8" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A102" s="1">
         <v>43542</v>
       </c>
@@ -4729,7 +4729,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="125" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:8" ht="116" x14ac:dyDescent="0.35">
       <c r="A125" s="1">
         <v>43984</v>
       </c>
@@ -5145,7 +5145,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="141" spans="1:8" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:8" ht="174" x14ac:dyDescent="0.35">
       <c r="A141" s="1">
         <v>44307</v>
       </c>
@@ -5353,7 +5353,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="149" spans="1:8" ht="232" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:8" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A149" s="1">
         <v>44474</v>
       </c>
@@ -5457,7 +5457,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="153" spans="1:8" ht="261" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:8" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A153" s="1">
         <v>45181</v>
       </c>
@@ -5613,7 +5613,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="159" spans="1:8" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:8" ht="145" x14ac:dyDescent="0.35">
       <c r="A159" s="1">
         <v>45750</v>
       </c>
@@ -6003,7 +6003,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="174" spans="1:8" ht="145" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:8" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A174" s="1">
         <v>42001</v>
       </c>
@@ -6731,7 +6731,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="202" spans="1:8" ht="232" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:8" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A202" s="1">
         <v>43203</v>
       </c>
@@ -7147,7 +7147,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="218" spans="1:8" ht="319" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:8" ht="333.5" x14ac:dyDescent="0.35">
       <c r="A218" s="1">
         <v>43951</v>
       </c>
@@ -7225,7 +7225,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="221" spans="1:8" ht="145" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:8" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A221" s="1">
         <v>43996</v>
       </c>
@@ -7355,7 +7355,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="226" spans="1:8" ht="290" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:8" ht="304.5" x14ac:dyDescent="0.35">
       <c r="A226" s="1">
         <v>44054</v>
       </c>
@@ -7745,7 +7745,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="241" spans="1:8" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:8" ht="174" x14ac:dyDescent="0.35">
       <c r="A241" s="1">
         <v>44398</v>
       </c>
@@ -8083,7 +8083,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="254" spans="1:8" ht="174" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:8" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A254" s="1">
         <v>44727</v>
       </c>
@@ -8629,7 +8629,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="275" spans="1:8" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:8" ht="145" x14ac:dyDescent="0.35">
       <c r="A275" s="1">
         <v>44986</v>
       </c>
@@ -8681,7 +8681,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="277" spans="1:8" ht="232" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:8" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A277" s="1">
         <v>45000</v>
       </c>
@@ -8785,7 +8785,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="281" spans="1:8" ht="290" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:8" ht="304.5" x14ac:dyDescent="0.35">
       <c r="A281" s="1">
         <v>45040</v>
       </c>
@@ -8837,7 +8837,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="283" spans="1:8" ht="348" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:8" ht="362.5" x14ac:dyDescent="0.35">
       <c r="A283" s="1">
         <v>45063</v>
       </c>
@@ -8964,7 +8964,7 @@
         <v>1</v>
       </c>
       <c r="H287" t="s">
-        <v>236</v>
+        <v>359</v>
       </c>
     </row>
     <row r="288" spans="1:8" ht="409.5" x14ac:dyDescent="0.35">
@@ -9071,7 +9071,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="292" spans="1:8" ht="275.5" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:8" ht="290" x14ac:dyDescent="0.35">
       <c r="A292" s="1">
         <v>45154</v>
       </c>
@@ -9175,7 +9175,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="296" spans="1:8" ht="304.5" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:8" ht="319" x14ac:dyDescent="0.35">
       <c r="A296" s="1">
         <v>45250</v>
       </c>
@@ -9383,7 +9383,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="304" spans="1:8" ht="304.5" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:8" ht="319" x14ac:dyDescent="0.35">
       <c r="A304" s="1">
         <v>45338</v>
       </c>
@@ -9487,7 +9487,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="308" spans="1:8" ht="217.5" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:8" ht="232" x14ac:dyDescent="0.35">
       <c r="A308" s="1">
         <v>45349</v>
       </c>
@@ -9877,7 +9877,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="323" spans="1:8" ht="377" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:8" ht="391.5" x14ac:dyDescent="0.35">
       <c r="A323" s="1">
         <v>45596</v>
       </c>
@@ -10137,7 +10137,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="333" spans="1:8" ht="217.5" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:8" ht="232" x14ac:dyDescent="0.35">
       <c r="A333" s="1">
         <v>45744</v>
       </c>
@@ -10267,7 +10267,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="338" spans="1:8" ht="275.5" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:8" ht="290" x14ac:dyDescent="0.35">
       <c r="A338" s="1">
         <v>45798</v>
       </c>

</xml_diff>